<commit_message>
refactoring, added numpy as dev package
</commit_message>
<xml_diff>
--- a/tests/datastructure/variable_definition.xlsx
+++ b/tests/datastructure/variable_definition.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="136">
   <si>
     <t xml:space="preserve">VaribleID</t>
   </si>
@@ -46,12 +46,12 @@
     <t xml:space="preserve">VariableDefaulValue</t>
   </si>
   <si>
+    <t xml:space="preserve">VariableLowerBound</t>
+  </si>
+  <si>
     <t xml:space="preserve">VariableUpperBound</t>
   </si>
   <si>
-    <t xml:space="preserve">VariableLowerBound</t>
-  </si>
-  <si>
     <t xml:space="preserve">Potentiaalberekening</t>
   </si>
   <si>
@@ -76,6 +76,9 @@
     <t xml:space="preserve">Input</t>
   </si>
   <si>
+    <t xml:space="preserve">none, deterministic</t>
+  </si>
+  <si>
     <t xml:space="preserve">input</t>
   </si>
   <si>
@@ -118,6 +121,12 @@
     <t xml:space="preserve">Geschematiseerde top van het zak in het vak</t>
   </si>
   <si>
+    <t xml:space="preserve">normal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">_stdev</t>
+  </si>
+  <si>
     <t xml:space="preserve">gamma_sat_deklaag</t>
   </si>
   <si>
@@ -127,6 +136,9 @@
     <t xml:space="preserve">kN/m^3</t>
   </si>
   <si>
+    <t xml:space="preserve">lognormal, shift 10</t>
+  </si>
+  <si>
     <t xml:space="preserve">D_deklaag</t>
   </si>
   <si>
@@ -136,6 +148,9 @@
     <t xml:space="preserve">Calculated</t>
   </si>
   <si>
+    <t xml:space="preserve">normal, by functional design &gt;0,1 m</t>
+  </si>
+  <si>
     <t xml:space="preserve">gamma_w</t>
   </si>
   <si>
@@ -154,6 +169,12 @@
     <t xml:space="preserve">m^2/dag</t>
   </si>
   <si>
+    <t xml:space="preserve">lognormal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">_vc</t>
+  </si>
+  <si>
     <t xml:space="preserve">D_wvp</t>
   </si>
   <si>
@@ -230,6 +251,9 @@
   </si>
   <si>
     <t xml:space="preserve">Buitenwaterstand</t>
+  </si>
+  <si>
+    <t xml:space="preserve">extreme value of CDF</t>
   </si>
   <si>
     <t xml:space="preserve">eta</t>
@@ -410,8 +434,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="#,##0.00"/>
+    <numFmt numFmtId="166" formatCode="0.00E+00"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -500,7 +526,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -519,6 +545,18 @@
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -713,7 +751,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N50"/>
+  <dimension ref="A1:O50"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.76"/>
@@ -726,10 +764,10 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="21.47"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="1" width="22.02"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="22.16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="16.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="16.89"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="17.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="17.85"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="15" style="1" width="11.53"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="16" style="1" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -789,16 +827,26 @@
       <c r="E2" s="3" t="s">
         <v>17</v>
       </c>
+      <c r="F2" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="I2" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="J2" s="5" t="n">
+        <v>2000</v>
+      </c>
       <c r="K2" s="3" t="s">
-        <v>18</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="O2" s="6"/>
     </row>
     <row r="3" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>16</v>
@@ -806,16 +854,24 @@
       <c r="E3" s="3" t="s">
         <v>17</v>
       </c>
+      <c r="F3" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="I3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" s="5"/>
       <c r="K3" s="3" t="s">
-        <v>18</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="O3" s="6"/>
     </row>
     <row r="4" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>16</v>
@@ -823,16 +879,24 @@
       <c r="E4" s="3" t="s">
         <v>17</v>
       </c>
+      <c r="F4" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="I4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="5"/>
       <c r="K4" s="3" t="s">
-        <v>18</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="O4" s="6"/>
     </row>
     <row r="5" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>16</v>
@@ -840,120 +904,202 @@
       <c r="E5" s="3" t="s">
         <v>17</v>
       </c>
+      <c r="F5" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="I5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="5" t="n">
+        <v>5000</v>
+      </c>
       <c r="K5" s="3" t="s">
-        <v>18</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="O5" s="6"/>
     </row>
     <row r="6" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>17</v>
       </c>
+      <c r="F6" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="I6" s="5" t="n">
+        <v>-4</v>
+      </c>
+      <c r="J6" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="O6" s="6"/>
     </row>
     <row r="7" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D7" s="3" t="s">
         <v>28</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>27</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>17</v>
       </c>
+      <c r="F7" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="I7" s="5"/>
+      <c r="J7" s="5"/>
       <c r="K7" s="3" t="s">
-        <v>18</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="O7" s="6"/>
     </row>
     <row r="8" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>17</v>
       </c>
+      <c r="F8" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="I8" s="5" t="n">
+        <v>-18</v>
+      </c>
+      <c r="J8" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="O8" s="6"/>
     </row>
     <row r="9" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="3" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>17</v>
       </c>
+      <c r="F9" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="I9" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="J9" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="O9" s="6"/>
     </row>
     <row r="10" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="3" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>16</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>37</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I10" s="5" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="J10" s="5"/>
+      <c r="O10" s="6"/>
     </row>
     <row r="11" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="3" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>40</v>
-      </c>
+        <v>45</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="H11" s="3" t="n">
+        <v>9.81</v>
+      </c>
+      <c r="I11" s="5"/>
+      <c r="J11" s="5"/>
+      <c r="O11" s="6"/>
     </row>
     <row r="12" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="3" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>17</v>
       </c>
+      <c r="F12" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="I12" s="5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="J12" s="5" t="n">
+        <v>4000</v>
+      </c>
       <c r="K12" s="3" t="s">
-        <v>18</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="O12" s="6"/>
     </row>
     <row r="13" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="3" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="D13" s="3" t="s">
         <v>16</v>
@@ -961,27 +1107,47 @@
       <c r="E13" s="3" t="s">
         <v>17</v>
       </c>
+      <c r="F13" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="I13" s="5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="J13" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="O13" s="6"/>
     </row>
     <row r="14" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="3" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>37</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="I14" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="J14" s="5" t="n">
+        <v>110</v>
+      </c>
+      <c r="O14" s="6"/>
     </row>
     <row r="15" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="3" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="D15" s="3" t="s">
         <v>16</v>
@@ -989,511 +1155,710 @@
       <c r="E15" s="3" t="s">
         <v>17</v>
       </c>
+      <c r="F15" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="I15" s="7" t="n">
+        <v>0.00015</v>
+      </c>
+      <c r="J15" s="7" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="O15" s="6"/>
     </row>
     <row r="16" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="3" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>17</v>
       </c>
+      <c r="F16" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="I16" s="5"/>
+      <c r="J16" s="5"/>
       <c r="K16" s="3" t="s">
-        <v>18</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="O16" s="6"/>
     </row>
     <row r="17" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="3" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>56</v>
-      </c>
+        <v>63</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="I17" s="5"/>
+      <c r="J17" s="5"/>
       <c r="K17" s="3" t="s">
-        <v>18</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="O17" s="6"/>
     </row>
     <row r="18" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="3" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>17</v>
       </c>
+      <c r="F18" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="I18" s="5"/>
+      <c r="J18" s="5"/>
+      <c r="O18" s="6"/>
     </row>
     <row r="19" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="3" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="E19" s="3" t="s">
         <v>17</v>
       </c>
+      <c r="F19" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="I19" s="5"/>
+      <c r="J19" s="5"/>
+      <c r="O19" s="6"/>
     </row>
     <row r="20" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="3" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>17</v>
       </c>
+      <c r="F20" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="I20" s="5"/>
+      <c r="J20" s="5"/>
+      <c r="O20" s="6"/>
     </row>
     <row r="21" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="3" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>40</v>
-      </c>
+        <v>45</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="H21" s="5" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="I21" s="5"/>
+      <c r="J21" s="5"/>
+      <c r="O21" s="6"/>
     </row>
     <row r="22" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D22" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="C22" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="D22" s="3" t="s">
-        <v>59</v>
-      </c>
       <c r="E22" s="3" t="s">
-        <v>40</v>
-      </c>
+        <v>45</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="H22" s="5" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="I22" s="5"/>
+      <c r="J22" s="5"/>
+      <c r="O22" s="6"/>
     </row>
     <row r="23" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="3" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E23" s="3" t="s">
         <v>17</v>
       </c>
+      <c r="F23" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="I23" s="5"/>
+      <c r="J23" s="5"/>
       <c r="K23" s="3" t="s">
-        <v>18</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="O23" s="6"/>
     </row>
     <row r="24" s="3" customFormat="true" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="3" t="s">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>40</v>
-      </c>
+        <v>45</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="H24" s="3" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="I24" s="5"/>
+      <c r="J24" s="5"/>
+      <c r="O24" s="6"/>
     </row>
     <row r="25" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="3" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>37</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="I25" s="5"/>
+      <c r="J25" s="5"/>
       <c r="K25" s="3" t="s">
-        <v>74</v>
-      </c>
+        <v>82</v>
+      </c>
+      <c r="O25" s="6"/>
     </row>
     <row r="26" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="3" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>37</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="I26" s="5"/>
+      <c r="J26" s="5"/>
       <c r="K26" s="3" t="s">
-        <v>74</v>
-      </c>
+        <v>82</v>
+      </c>
+      <c r="O26" s="6"/>
     </row>
     <row r="27" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="3" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>37</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="I27" s="5"/>
+      <c r="J27" s="5"/>
+      <c r="O27" s="6"/>
     </row>
     <row r="28" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="3" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="D28" s="3" t="s">
         <v>16</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>37</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="I28" s="5"/>
+      <c r="J28" s="5"/>
+      <c r="O28" s="6"/>
     </row>
     <row r="29" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="3" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>40</v>
-      </c>
+        <v>45</v>
+      </c>
+      <c r="F29" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="H29" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="I29" s="5"/>
+      <c r="J29" s="5"/>
+      <c r="O29" s="6"/>
     </row>
     <row r="30" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="3" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="D30" s="3" t="s">
         <v>16</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>40</v>
-      </c>
+        <v>45</v>
+      </c>
+      <c r="F30" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="H30" s="7" t="n">
+        <v>0.000208</v>
+      </c>
+      <c r="I30" s="5"/>
+      <c r="J30" s="5"/>
+      <c r="O30" s="6"/>
     </row>
     <row r="31" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="3" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>40</v>
-      </c>
+        <v>45</v>
+      </c>
+      <c r="F31" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="H31" s="3" t="n">
+        <v>9.81</v>
+      </c>
+      <c r="I31" s="5"/>
+      <c r="J31" s="5"/>
+      <c r="O31" s="6"/>
     </row>
     <row r="32" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="3" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>40</v>
-      </c>
+        <v>45</v>
+      </c>
+      <c r="F32" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="H32" s="7" t="n">
+        <v>1.33E-006</v>
+      </c>
+      <c r="I32" s="5"/>
+      <c r="J32" s="5"/>
+      <c r="O32" s="6"/>
     </row>
     <row r="33" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="3" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>40</v>
-      </c>
+        <v>45</v>
+      </c>
+      <c r="F33" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="H33" s="5" t="n">
+        <v>26</v>
+      </c>
+      <c r="I33" s="5"/>
+      <c r="J33" s="5"/>
+      <c r="O33" s="6"/>
     </row>
     <row r="34" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="3" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="D34" s="3" t="s">
         <v>16</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>37</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="I34" s="5"/>
+      <c r="J34" s="5"/>
+      <c r="O34" s="6"/>
     </row>
     <row r="35" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="3" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="D35" s="3" t="s">
         <v>16</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>37</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="I35" s="5"/>
+      <c r="J35" s="5"/>
+      <c r="O35" s="6"/>
     </row>
     <row r="36" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="3" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>37</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="I36" s="5"/>
+      <c r="J36" s="5"/>
+      <c r="O36" s="6"/>
     </row>
     <row r="37" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="3" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="D37" s="3" t="s">
         <v>16</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>37</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="I37" s="5"/>
+      <c r="J37" s="5"/>
+      <c r="O37" s="6"/>
     </row>
     <row r="38" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="3" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>37</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="I38" s="5"/>
+      <c r="J38" s="5"/>
+      <c r="O38" s="6"/>
     </row>
     <row r="39" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="3" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>37</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="I39" s="5"/>
+      <c r="J39" s="5"/>
+      <c r="O39" s="6"/>
     </row>
     <row r="40" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="3" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>37</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="I40" s="5"/>
+      <c r="J40" s="5"/>
+      <c r="O40" s="6"/>
     </row>
     <row r="41" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="3" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>37</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="I41" s="5"/>
+      <c r="J41" s="5"/>
+      <c r="O41" s="6"/>
     </row>
     <row r="42" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="3" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="D42" s="3" t="s">
         <v>16</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>37</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="I42" s="5"/>
+      <c r="J42" s="5"/>
+      <c r="O42" s="6"/>
     </row>
     <row r="43" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="3" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="D43" s="3" t="s">
         <v>16</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>37</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="I43" s="5"/>
+      <c r="J43" s="5"/>
+      <c r="O43" s="6"/>
     </row>
     <row r="44" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="3" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="D44" s="3" t="s">
         <v>16</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>37</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="I44" s="5"/>
+      <c r="J44" s="5"/>
+      <c r="O44" s="6"/>
     </row>
     <row r="45" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="3" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="D45" s="3" t="s">
         <v>16</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>37</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="I45" s="5"/>
+      <c r="J45" s="5"/>
+      <c r="O45" s="6"/>
     </row>
     <row r="46" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="3" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="D46" s="3" t="s">
         <v>16</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>37</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="I46" s="5"/>
+      <c r="J46" s="5"/>
+      <c r="O46" s="6"/>
     </row>
     <row r="47" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B47" s="3" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="D47" s="3" t="s">
         <v>16</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>37</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="I47" s="5"/>
+      <c r="J47" s="5"/>
+      <c r="O47" s="6"/>
     </row>
     <row r="48" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B48" s="3" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>37</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="I48" s="5"/>
+      <c r="J48" s="5"/>
+      <c r="O48" s="6"/>
     </row>
     <row r="49" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="3" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>37</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="I49" s="5"/>
+      <c r="J49" s="5"/>
+      <c r="O49" s="6"/>
     </row>
     <row r="50" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="3" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>37</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="I50" s="5"/>
+      <c r="J50" s="5"/>
+      <c r="O50" s="6"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>